<commit_message>
Address ELC evidence completeness findings
</commit_message>
<xml_diff>
--- a/2.RCM/ELC_RCM.xlsx
+++ b/2.RCM/ELC_RCM.xlsx
@@ -744,7 +744,7 @@
       </c>
       <c r="K6" s="6" t="inlineStr">
         <is>
-          <t>HRISの受講・受領確認ログを母集団として入手し、対象者数、完了者数、未了者ゼロ又は督促完了を確認する。</t>
+          <t>HRISの対象者別受領確認ログを母集団として入手し、集計行の対象者数522名と個票明細522件、受領確認済件数522件が一致していることを確認する。</t>
         </is>
       </c>
       <c r="L6" s="6" t="inlineStr">
@@ -836,7 +836,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>職務権限・組織体制_年次レビュー_FY2025.csv; 規程_職務権限規程_R18.pdf; employees.xlsx; company_profile.md</t>
+          <t>財務報告責任者一覧_承認証跡_FY2025.csv; 職務権限・組織体制_年次レビュー_FY2025.csv; 規程_職務権限規程_R18.pdf; employees.xlsx; company_profile.md</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Convert ELC company profile evidence to PDF
</commit_message>
<xml_diff>
--- a/2.RCM/ELC_RCM.xlsx
+++ b/2.RCM/ELC_RCM.xlsx
@@ -836,7 +836,7 @@
       </c>
       <c r="L7" s="6" t="inlineStr">
         <is>
-          <t>財務報告責任者一覧_承認証跡_FY2025.csv; 職務権限・組織体制_年次レビュー_FY2025.csv; 規程_職務権限規程_R18.pdf; employees.xlsx; company_profile.md</t>
+          <t>財務報告責任者一覧_承認証跡_FY2025.csv; 職務権限・組織体制_年次レビュー_FY2025.csv; 規程_職務権限規程_R18.pdf; employees.xlsx; company_profile.pdf</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
@@ -1097,7 +1097,7 @@
       </c>
       <c r="L10" s="6" t="inlineStr">
         <is>
-          <t>規程・業務手順_年次レビュー台帳_FY2025.xlsx; company_profile.md</t>
+          <t>規程・業務手順_年次レビュー台帳_FY2025.xlsx; company_profile.pdf</t>
         </is>
       </c>
       <c r="M10" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Address ELC-010 and ELC-012 evidence gaps
</commit_message>
<xml_diff>
--- a/2.RCM/ELC_RCM.xlsx
+++ b/2.RCM/ELC_RCM.xlsx
@@ -1410,7 +1410,7 @@
       </c>
       <c r="E14" s="6" t="inlineStr">
         <is>
-          <t>内部監査室は財務報告リスク評価に基づき年次内部監査計画を策定し、ELC、PLC、ITGC、ITAC、FCRPの整備・運用評価を実施する。発見事項はCFO、代表取締役、監査等委員会へ報告し、是正をフォローする。</t>
+          <t>内部監査室は財務報告リスク評価に基づき年次内部監査計画を策定し、ELC、PLC、ITGC、ITAC、FCRPの評価対象、実施時期、担当者を定めて整備・運用評価を実施する。発見事項はCFO、代表取締役、監査等委員会へ報告し、是正をフォローする。</t>
         </is>
       </c>
       <c r="F14" s="5" t="inlineStr">
@@ -1584,7 +1584,7 @@
       </c>
       <c r="E16" s="6" t="inlineStr">
         <is>
-          <t>情報システム部は年次IT計画、情報セキュリティ方針、ITGC評価範囲、外部委託先SOC1報告書及びCUEC対応状況をレビューし、重要なITリスク及び委託先不備を経営会議又は取締役会へ報告する。</t>
+          <t>情報システム部は年次IT計画、情報セキュリティ方針、ITGC評価範囲、外部委託先SOC1報告書及びCUEC対応状況をレビューする。CUECごとに自社側統制、責任者、対応状況、証跡、報告記録を台帳で管理し、重要なITリスク及び委託先不備を経営会議又は取締役会へ報告する。</t>
         </is>
       </c>
       <c r="F16" s="5" t="inlineStr">
@@ -1609,12 +1609,12 @@
       </c>
       <c r="J16" s="6" t="inlineStr">
         <is>
-          <t>情報セキュリティ基本方針、IT関連規程、外部委託管理規程を閲覧し、IT計画、ITリスク、委託先報告書、CUEC対応のレビュー要件が定義されていることを確認する。</t>
+          <t>情報セキュリティ基本方針、IT関連規程、外部委託管理規程を閲覧し、IT計画、ITリスク、委託先報告書、CUEC対応のレビュー要件及び経営報告要件が定義されていることを確認する。</t>
         </is>
       </c>
       <c r="K16" s="6" t="inlineStr">
         <is>
-          <t>ITガバナンス・外部委託先レビュー台帳とSOC1報告書を閲覧し、財務報告関連ITリスク、SOC1例外、CUEC対応、経営報告が記録されていることを確認する。</t>
+          <t>ITガバナンス・外部委託先レビュー台帳とSOC1報告書を閲覧し、財務報告関連ITリスク、SOC1例外、CUECごとの自社側統制ID・責任者・対応状況・証跡、及び経営報告ログが追跡可能に記録されていることを確認する。</t>
         </is>
       </c>
       <c r="L16" s="6" t="inlineStr">

</xml_diff>

<commit_message>
Normalize ELC evidence mappings
</commit_message>
<xml_diff>
--- a/2.RCM/ELC_RCM.xlsx
+++ b/2.RCM/ELC_RCM.xlsx
@@ -1184,7 +1184,7 @@
       </c>
       <c r="L11" s="6" t="inlineStr">
         <is>
-          <t>SAP_PeriodClose_JobLog_FY2025.csv; 財務報告連絡会_議事メモ_2025年度Q4.md</t>
+          <t>SAP_PeriodClose_JobLog_FY2025.csv; 財務報告連絡会_議事メモ_2025年度Q4.pdf</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
@@ -1358,7 +1358,7 @@
       </c>
       <c r="L13" s="6" t="inlineStr">
         <is>
-          <t>財務報告連絡会_開催実績_FY2025.csv; 財務報告連絡会_議事メモ_2025年度Q4.md</t>
+          <t>財務報告連絡会_開催実績_FY2025.csv; 財務報告連絡会_議事メモ_2025年度Q4.pdf</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">

</xml_diff>